<commit_message>
changing things and work
</commit_message>
<xml_diff>
--- a/input/ampq.xlsx
+++ b/input/ampq.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mój dysk\AMPQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E931D242-DAF6-4694-ABBA-85209D6A6CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF1DDE1-C69F-4800-849F-DE590D0B04B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3465E9D8-2616-4A3B-901D-12D504620602}"/>
   </bookViews>
@@ -31,12 +31,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="134">
   <si>
     <t>QTY</t>
   </si>
@@ -68,9 +71,6 @@
     <t>Xiaomi 33W Power Bank 10000mAh (Integrated Cable) BHR9341GL</t>
   </si>
   <si>
-    <t>Xiaomi Compact Hair Dryer H101 White EU BHR7475EU</t>
-  </si>
-  <si>
     <t>Xiaomi Electric Shaver S101 EU BHR7456EU</t>
   </si>
   <si>
@@ -236,9 +236,6 @@
     <t>Google Pixel 9a 8/128GB Black GA05769-GB</t>
   </si>
   <si>
-    <t>Xiaomi Redmi A5 4G 3/64GB Midnight Black MZB0JSEEU</t>
-  </si>
-  <si>
     <t>Xiaomi Redmi 15C 4G NFC 8/256GB Midnight Black MZB0KOCEU</t>
   </si>
   <si>
@@ -317,9 +314,6 @@
     <t>Xiaomi Semi-automatic Espresso Machine EU BHR9798EU</t>
   </si>
   <si>
-    <t>Xiaomi Smart Air Purifier 4 Pro EU BHR5056EU</t>
-  </si>
-  <si>
     <t>Xiaomi Smart Standing Fan 2 Pro EU BHR5856EU</t>
   </si>
   <si>
@@ -365,9 +359,6 @@
     <t>Xiaomi Super Slim Magnetic Power Bank 5000 Gold BHR08PLGL</t>
   </si>
   <si>
-    <t>Xiaomi UltraThin Magnetic Power Bank 5000 15W Glacier Silver BHR08Z2GL</t>
-  </si>
-  <si>
     <t>Remington TouchTech Beard Trimmer EU MB4700</t>
   </si>
   <si>
@@ -407,9 +398,6 @@
     <t>Xiaomi Sound Outdoor 30W Red QBH4263GL</t>
   </si>
   <si>
-    <t>(incoming 23.03)</t>
-  </si>
-  <si>
     <t>Samsung S24 8GB/256GB Purple SM-S921BZVGEUE</t>
   </si>
   <si>
@@ -449,10 +437,10 @@
     <t>Samsung Galaxy S26 Ultra 512GB White SM-S948BZWGEUE</t>
   </si>
   <si>
-    <t>Remington AIRvive Haartrockner</t>
-  </si>
-  <si>
     <t>(incoming 26.03)</t>
+  </si>
+  <si>
+    <t>Apple iPhone 17 256GB Sage MG6N4HX/A</t>
   </si>
 </sst>
 </file>
@@ -842,7 +830,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A360796-7343-4130-90EE-C427191F85B0}">
-  <dimension ref="A1:F130"/>
+  <dimension ref="A1:F126"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -878,10 +866,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="C2" t="str">
-        <f t="shared" ref="C2:C61" si="0">MID(B2,FIND("@",SUBSTITUTE(B2," ","@",LEN(B2)-LEN(SUBSTITUTE(B2," ",""))))+1,LEN(B2))</f>
+        <f t="shared" ref="C2:C65" si="0">MID(B2,FIND("@",SUBSTITUTE(B2," ","@",LEN(B2)-LEN(SUBSTITUTE(B2," ",""))))+1,LEN(B2))</f>
         <v>MG6J4HX/A</v>
       </c>
       <c r="D2" s="3">
@@ -899,7 +887,7 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C3" t="str">
         <f t="shared" si="0"/>
@@ -920,7 +908,7 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C4" t="str">
         <f t="shared" si="0"/>
@@ -941,7 +929,7 @@
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="0"/>
@@ -959,20 +947,20 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>420</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>133</v>
       </c>
       <c r="C6" t="str">
         <f t="shared" si="0"/>
-        <v>MXN43ZM/A</v>
+        <v>MG6N4HX/A</v>
       </c>
       <c r="D6" s="3">
-        <v>195949690457</v>
+        <v>195950644258</v>
       </c>
       <c r="E6">
-        <v>61</v>
+        <v>739</v>
       </c>
       <c r="F6" t="s">
         <v>6</v>
@@ -980,20 +968,20 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>55</v>
+        <v>410</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="0"/>
-        <v>GA05769-GB</v>
+        <v>MXN43ZM/A</v>
       </c>
       <c r="D7" s="3">
-        <v>840353922273</v>
+        <v>195949690457</v>
       </c>
       <c r="E7">
-        <v>299</v>
+        <v>61</v>
       </c>
       <c r="F7" t="s">
         <v>6</v>
@@ -1001,19 +989,20 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>125</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>58</v>
+        <v>64</v>
+      </c>
+      <c r="C8" t="str">
+        <f t="shared" si="0"/>
+        <v>GA05769-GB</v>
       </c>
       <c r="D8" s="3">
-        <v>6941764469662</v>
+        <v>840353922273</v>
       </c>
       <c r="E8">
-        <v>75</v>
+        <v>299</v>
       </c>
       <c r="F8" t="s">
         <v>6</v>
@@ -1024,13 +1013,14 @@
         <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>126</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>58</v>
+        <v>120</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="0"/>
+        <v>RMX5313</v>
       </c>
       <c r="D9" s="3">
-        <v>6941764469655</v>
+        <v>6941764469662</v>
       </c>
       <c r="E9">
         <v>75</v>
@@ -1041,19 +1031,20 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
+        <v>40</v>
+      </c>
+      <c r="B10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C10" t="str">
+        <f t="shared" si="0"/>
+        <v>RMX5313</v>
+      </c>
+      <c r="D10" s="3">
+        <v>6941764469655</v>
+      </c>
+      <c r="E10">
         <v>75</v>
-      </c>
-      <c r="B10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="3">
-        <v>6941764482890</v>
-      </c>
-      <c r="E10">
-        <v>359</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
@@ -1061,19 +1052,20 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="B11" t="s">
-        <v>127</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>58</v>
+        <v>128</v>
+      </c>
+      <c r="C11" t="str">
+        <f t="shared" si="0"/>
+        <v>Grey</v>
       </c>
       <c r="D11" s="3">
-        <v>6941764466920</v>
+        <v>6941764482890</v>
       </c>
       <c r="E11">
-        <v>379</v>
+        <v>359</v>
       </c>
       <c r="F11" t="s">
         <v>6</v>
@@ -1081,20 +1073,20 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>122</v>
       </c>
       <c r="C12" t="str">
         <f t="shared" si="0"/>
-        <v>SM-A366BZABEUE</v>
+        <v>Black</v>
       </c>
       <c r="D12" s="3">
-        <v>8806095984261</v>
+        <v>6941764466920</v>
       </c>
       <c r="E12">
-        <v>195</v>
+        <v>379</v>
       </c>
       <c r="F12" t="s">
         <v>6</v>
@@ -1102,20 +1094,20 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>115</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>124</v>
+        <v>35</v>
       </c>
       <c r="C13" t="str">
         <f t="shared" si="0"/>
-        <v>SM-S921BZVGEUE</v>
+        <v>SM-A366BZABEUE</v>
       </c>
       <c r="D13" s="3">
-        <v>8806095299662</v>
+        <v>8806095984261</v>
       </c>
       <c r="E13">
-        <v>479</v>
+        <v>195</v>
       </c>
       <c r="F13" t="s">
         <v>6</v>
@@ -1123,20 +1115,20 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="B14" t="s">
-        <v>59</v>
+        <v>119</v>
       </c>
       <c r="C14" t="str">
         <f t="shared" si="0"/>
-        <v>SM-S942BZKHEUE</v>
+        <v>SM-S921BZVGEUE</v>
       </c>
       <c r="D14" s="3">
-        <v>8806097827405</v>
+        <v>8806095299662</v>
       </c>
       <c r="E14">
-        <v>672</v>
+        <v>479</v>
       </c>
       <c r="F14" t="s">
         <v>6</v>
@@ -1144,20 +1136,20 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="B15" t="s">
-        <v>135</v>
+        <v>58</v>
       </c>
       <c r="C15" t="str">
         <f t="shared" si="0"/>
-        <v>SM-S948BZKGEUE</v>
+        <v>SM-S942BZKHEUE</v>
       </c>
       <c r="D15" s="3">
-        <v>8806097827177</v>
+        <v>8806097827405</v>
       </c>
       <c r="E15">
-        <v>949</v>
+        <v>672</v>
       </c>
       <c r="F15" t="s">
         <v>6</v>
@@ -1165,10 +1157,10 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B16" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C16" t="str">
         <f t="shared" si="0"/>
@@ -1181,7 +1173,7 @@
         <v>949</v>
       </c>
       <c r="F16" t="s">
-        <v>138</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1189,41 +1181,41 @@
         <v>50</v>
       </c>
       <c r="B17" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C17" t="str">
         <f t="shared" si="0"/>
-        <v>SM-S948BZWGEUE</v>
+        <v>SM-S948BZKGEUE</v>
       </c>
       <c r="D17" s="3">
-        <v>8806097826880</v>
+        <v>8806097827177</v>
       </c>
       <c r="E17">
         <v>949</v>
       </c>
       <c r="F17" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>131</v>
       </c>
       <c r="C18" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0JSEEU</v>
+        <v>SM-S948BZWGEUE</v>
       </c>
       <c r="D18" s="3">
-        <v>6932554425104</v>
+        <v>8806097826880</v>
       </c>
       <c r="E18">
-        <v>61</v>
+        <v>949</v>
       </c>
       <c r="F18" t="s">
-        <v>6</v>
+        <v>132</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1231,7 +1223,7 @@
         <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C19" t="str">
         <f t="shared" si="0"/>
@@ -1252,7 +1244,7 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C20" t="str">
         <f t="shared" si="0"/>
@@ -1273,7 +1265,7 @@
         <v>5</v>
       </c>
       <c r="B21" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C21" t="str">
         <f t="shared" si="0"/>
@@ -1294,7 +1286,7 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C22" t="str">
         <f t="shared" si="0"/>
@@ -1315,7 +1307,7 @@
         <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C23" t="str">
         <f t="shared" si="0"/>
@@ -1336,7 +1328,7 @@
         <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C24" t="str">
         <f t="shared" si="0"/>
@@ -1357,7 +1349,7 @@
         <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C25" t="str">
         <f t="shared" si="0"/>
@@ -1378,7 +1370,7 @@
         <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="C26" t="str">
         <f t="shared" si="0"/>
@@ -1399,7 +1391,7 @@
         <v>5</v>
       </c>
       <c r="B27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C27" t="str">
         <f t="shared" si="0"/>
@@ -1417,10 +1409,10 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B28" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C28" t="str">
         <f t="shared" si="0"/>
@@ -1441,7 +1433,7 @@
         <v>15</v>
       </c>
       <c r="B29" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C29" t="str">
         <f t="shared" si="0"/>
@@ -1462,10 +1454,10 @@
         <v>4</v>
       </c>
       <c r="B30" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D30" s="3">
         <v>6932554478001</v>
@@ -1482,10 +1474,10 @@
         <v>5</v>
       </c>
       <c r="B31" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D31" s="3">
         <v>6932554478100</v>
@@ -1502,10 +1494,10 @@
         <v>4</v>
       </c>
       <c r="B32" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D32" s="3">
         <v>6932554477998</v>
@@ -1522,7 +1514,7 @@
         <v>4</v>
       </c>
       <c r="B33" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C33" t="str">
         <f t="shared" si="0"/>
@@ -1543,7 +1535,7 @@
         <v>4</v>
       </c>
       <c r="B34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C34" t="str">
         <f t="shared" si="0"/>
@@ -1564,7 +1556,7 @@
         <v>5</v>
       </c>
       <c r="B35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C35" t="str">
         <f t="shared" si="0"/>
@@ -1585,7 +1577,7 @@
         <v>5</v>
       </c>
       <c r="B36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C36" t="str">
         <f t="shared" si="0"/>
@@ -1606,10 +1598,10 @@
         <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D37" s="3">
         <v>6932554480943</v>
@@ -1626,7 +1618,7 @@
         <v>10</v>
       </c>
       <c r="B38" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C38" t="str">
         <f t="shared" si="0"/>
@@ -1647,7 +1639,7 @@
         <v>10</v>
       </c>
       <c r="B39" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C39" t="str">
         <f t="shared" si="0"/>
@@ -1668,7 +1660,7 @@
         <v>9</v>
       </c>
       <c r="B40" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C40" t="str">
         <f t="shared" si="0"/>
@@ -1689,7 +1681,7 @@
         <v>10</v>
       </c>
       <c r="B41" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C41" t="str">
         <f t="shared" si="0"/>
@@ -1710,7 +1702,7 @@
         <v>10</v>
       </c>
       <c r="B42" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C42" t="str">
         <f t="shared" si="0"/>
@@ -1731,7 +1723,7 @@
         <v>10</v>
       </c>
       <c r="B43" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C43" t="str">
         <f t="shared" si="0"/>
@@ -1752,7 +1744,7 @@
         <v>10</v>
       </c>
       <c r="B44" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C44" t="str">
         <f t="shared" si="0"/>
@@ -1773,7 +1765,7 @@
         <v>15</v>
       </c>
       <c r="B45" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C45" t="str">
         <f t="shared" si="0"/>
@@ -1794,7 +1786,7 @@
         <v>120</v>
       </c>
       <c r="B46" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C46" t="str">
         <f t="shared" si="0"/>
@@ -1815,7 +1807,7 @@
         <v>50</v>
       </c>
       <c r="B47" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C47" t="str">
         <f t="shared" si="0"/>
@@ -1836,7 +1828,7 @@
         <v>25</v>
       </c>
       <c r="B48" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C48" t="str">
         <f t="shared" si="0"/>
@@ -1857,7 +1849,7 @@
         <v>55</v>
       </c>
       <c r="B49" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C49" t="str">
         <f t="shared" si="0"/>
@@ -1875,13 +1867,13 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="B50" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D50" s="3">
         <v>815820024071</v>
@@ -1898,7 +1890,7 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C51" t="str">
         <f t="shared" si="0"/>
@@ -1919,7 +1911,7 @@
         <v>15</v>
       </c>
       <c r="B52" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C52" t="str">
         <f t="shared" si="0"/>
@@ -1940,7 +1932,7 @@
         <v>75</v>
       </c>
       <c r="B53" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C53" t="str">
         <f t="shared" si="0"/>
@@ -1958,10 +1950,10 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>270</v>
+        <v>230</v>
       </c>
       <c r="B54" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C54" t="str">
         <f t="shared" si="0"/>
@@ -1982,7 +1974,7 @@
         <v>130</v>
       </c>
       <c r="B55" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C55" t="str">
         <f t="shared" si="0"/>
@@ -2003,7 +1995,7 @@
         <v>20</v>
       </c>
       <c r="B56" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C56" t="str">
         <f t="shared" si="0"/>
@@ -2021,10 +2013,10 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="B57" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C57" t="str">
         <f t="shared" si="0"/>
@@ -2045,7 +2037,7 @@
         <v>50</v>
       </c>
       <c r="B58" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C58" t="str">
         <f t="shared" si="0"/>
@@ -2066,7 +2058,7 @@
         <v>5</v>
       </c>
       <c r="B59" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C59" t="str">
         <f t="shared" si="0"/>
@@ -2087,7 +2079,7 @@
         <v>10</v>
       </c>
       <c r="B60" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C60" t="str">
         <f t="shared" si="0"/>
@@ -2108,7 +2100,7 @@
         <v>5</v>
       </c>
       <c r="B61" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C61" t="str">
         <f t="shared" si="0"/>
@@ -2129,10 +2121,10 @@
         <v>10</v>
       </c>
       <c r="B62" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C62" t="str">
-        <f t="shared" ref="C62:C120" si="1">MID(B62,FIND("@",SUBSTITUTE(B62," ","@",LEN(B62)-LEN(SUBSTITUTE(B62," ",""))))+1,LEN(B62))</f>
+        <f t="shared" si="0"/>
         <v>ES501EU</v>
       </c>
       <c r="D62" s="3">
@@ -2150,10 +2142,10 @@
         <v>15</v>
       </c>
       <c r="B63" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C63" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>ES701EU</v>
       </c>
       <c r="D63" s="3">
@@ -2171,10 +2163,10 @@
         <v>5</v>
       </c>
       <c r="B64" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C64" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>CB100EU</v>
       </c>
       <c r="D64" s="3">
@@ -2192,10 +2184,10 @@
         <v>5</v>
       </c>
       <c r="B65" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C65" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>TB301EU</v>
       </c>
       <c r="D65" s="3">
@@ -2213,10 +2205,10 @@
         <v>10</v>
       </c>
       <c r="B66" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C66" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="C66:C126" si="1">MID(B66,FIND("@",SUBSTITUTE(B66," ","@",LEN(B66)-LEN(SUBSTITUTE(B66," ",""))))+1,LEN(B66))</f>
         <v>QB3001EUS</v>
       </c>
       <c r="D66" s="3">
@@ -2231,13 +2223,13 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B67" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D67" s="3">
         <v>45496321529</v>
@@ -2254,7 +2246,7 @@
         <v>15</v>
       </c>
       <c r="B68" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C68" t="str">
         <f t="shared" si="1"/>
@@ -2275,7 +2267,7 @@
         <v>70</v>
       </c>
       <c r="B69" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C69" t="str">
         <f t="shared" si="1"/>
@@ -2296,7 +2288,7 @@
         <v>20</v>
       </c>
       <c r="B70" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C70" t="str">
         <f t="shared" si="1"/>
@@ -2317,10 +2309,10 @@
         <v>200</v>
       </c>
       <c r="B71" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D71" s="3">
         <v>6941764428546</v>
@@ -2337,10 +2329,10 @@
         <v>200</v>
       </c>
       <c r="B72" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D72" s="3">
         <v>6941764467194</v>
@@ -2354,13 +2346,13 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="B73" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D73" s="3">
         <v>6941764432994</v>
@@ -2377,10 +2369,10 @@
         <v>35</v>
       </c>
       <c r="B74" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D74" s="3">
         <v>6941764483408</v>
@@ -2397,7 +2389,7 @@
         <v>330</v>
       </c>
       <c r="B75" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C75" t="str">
         <f t="shared" si="1"/>
@@ -2418,7 +2410,7 @@
         <v>50</v>
       </c>
       <c r="B76" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C76" t="str">
         <f t="shared" si="1"/>
@@ -2436,19 +2428,20 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B77" t="s">
-        <v>137</v>
-      </c>
-      <c r="C77" s="5" t="s">
-        <v>58</v>
+        <v>107</v>
+      </c>
+      <c r="C77" t="str">
+        <f t="shared" si="1"/>
+        <v>CF9530F0</v>
       </c>
       <c r="D77" s="3">
-        <v>5038061174762</v>
+        <v>3121040062753</v>
       </c>
       <c r="E77">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="F77" t="s">
         <v>6</v>
@@ -2456,41 +2449,41 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="B78" t="s">
-        <v>111</v>
+        <v>23</v>
       </c>
       <c r="C78" t="str">
         <f t="shared" si="1"/>
-        <v>CF9530F0</v>
+        <v>EB-P3400XUEGEU</v>
       </c>
       <c r="D78" s="3">
-        <v>3121040062753</v>
+        <v>8806094682748</v>
       </c>
       <c r="E78">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F78" t="s">
-        <v>123</v>
+        <v>6</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="B79" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="C79" t="str">
         <f t="shared" si="1"/>
-        <v>EB-P3400XUEGEU</v>
+        <v>EI-T5600BBEGWW</v>
       </c>
       <c r="D79" s="3">
-        <v>8806094682748</v>
+        <v>8806095031415</v>
       </c>
       <c r="E79">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F79" t="s">
         <v>6</v>
@@ -2498,17 +2491,17 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="B80" t="s">
         <v>39</v>
       </c>
       <c r="C80" t="str">
         <f t="shared" si="1"/>
-        <v>EI-T5600BBEGWW</v>
+        <v>EI-T5600BWEGWW</v>
       </c>
       <c r="D80" s="3">
-        <v>8806095031415</v>
+        <v>8806095031408</v>
       </c>
       <c r="E80">
         <v>12</v>
@@ -2519,20 +2512,20 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>300</v>
+        <v>40</v>
       </c>
       <c r="B81" t="s">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="C81" t="str">
         <f t="shared" si="1"/>
-        <v>EI-T5600BWEGWW</v>
+        <v>SM-L310NZGAEUE</v>
       </c>
       <c r="D81" s="3">
-        <v>8806095031408</v>
+        <v>8806095660981</v>
       </c>
       <c r="E81">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="F81" t="s">
         <v>6</v>
@@ -2540,20 +2533,20 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="B82" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C82" t="str">
         <f t="shared" si="1"/>
-        <v>SM-L310NZGAEUE</v>
+        <v>SM-L310NZSAEUE</v>
       </c>
       <c r="D82" s="3">
-        <v>8806095660981</v>
+        <v>8806095660684</v>
       </c>
       <c r="E82">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F82" t="s">
         <v>6</v>
@@ -2561,20 +2554,20 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="B83" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C83" t="str">
         <f t="shared" si="1"/>
-        <v>SM-L310NZSAEUE</v>
+        <v>SM-L320NZSAEUE</v>
       </c>
       <c r="D83" s="3">
-        <v>8806095660684</v>
+        <v>8806097415756</v>
       </c>
       <c r="E83">
-        <v>136</v>
+        <v>165</v>
       </c>
       <c r="F83" t="s">
         <v>6</v>
@@ -2582,41 +2575,41 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="B84" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C84" t="str">
         <f t="shared" si="1"/>
-        <v>SM-L320NZSAEUE</v>
+        <v>PX250EUT</v>
       </c>
       <c r="D84" s="3">
-        <v>8806097415756</v>
+        <v>622356307024</v>
       </c>
       <c r="E84">
-        <v>167</v>
+        <v>125</v>
       </c>
       <c r="F84" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B85" t="s">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="C85" t="str">
         <f t="shared" si="1"/>
-        <v>PX250EUT</v>
+        <v>IW3612EU</v>
       </c>
       <c r="D85" s="3">
-        <v>622356307024</v>
+        <v>622356310352</v>
       </c>
       <c r="E85">
-        <v>125</v>
+        <v>205</v>
       </c>
       <c r="F85" t="s">
         <v>7</v>
@@ -2624,20 +2617,20 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B86" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C86" t="str">
         <f t="shared" si="1"/>
-        <v>IW3612EU</v>
+        <v>HD446SLEU</v>
       </c>
       <c r="D86" s="3">
-        <v>622356310352</v>
+        <v>622356306621</v>
       </c>
       <c r="E86">
-        <v>205</v>
+        <v>153</v>
       </c>
       <c r="F86" t="s">
         <v>7</v>
@@ -2645,20 +2638,20 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B87" t="s">
         <v>60</v>
       </c>
       <c r="C87" t="str">
         <f t="shared" si="1"/>
-        <v>HD446SLEU</v>
+        <v>S6003EU</v>
       </c>
       <c r="D87" s="3">
-        <v>622356306621</v>
+        <v>622356220743</v>
       </c>
       <c r="E87">
-        <v>153</v>
+        <v>65</v>
       </c>
       <c r="F87" t="s">
         <v>7</v>
@@ -2666,61 +2659,61 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="B88" t="s">
-        <v>61</v>
+        <v>108</v>
       </c>
       <c r="C88" t="str">
         <f t="shared" si="1"/>
-        <v>S6003EU</v>
+        <v>178236</v>
       </c>
       <c r="D88" s="3">
-        <v>622356220743</v>
+        <v>4023103254145</v>
       </c>
       <c r="E88">
-        <v>65</v>
+        <v>155</v>
       </c>
       <c r="F88" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B89" t="s">
-        <v>112</v>
-      </c>
-      <c r="C89" t="str">
-        <f t="shared" si="1"/>
-        <v>178236</v>
+        <v>109</v>
+      </c>
+      <c r="C89" s="5" t="s">
+        <v>57</v>
       </c>
       <c r="D89" s="3">
-        <v>4023103254145</v>
+        <v>4023103246584</v>
       </c>
       <c r="E89">
-        <v>155</v>
+        <v>17</v>
       </c>
       <c r="F89" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
-        <v>100</v>
+        <v>350</v>
       </c>
       <c r="B90" t="s">
-        <v>113</v>
-      </c>
-      <c r="C90" s="5" t="s">
-        <v>58</v>
+        <v>24</v>
+      </c>
+      <c r="C90" t="str">
+        <f t="shared" si="1"/>
+        <v>BHR6942EU</v>
       </c>
       <c r="D90" s="3">
-        <v>4023103246584</v>
+        <v>6941812708347</v>
       </c>
       <c r="E90">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="F90" t="s">
         <v>7</v>
@@ -2728,20 +2721,20 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91">
-        <v>350</v>
+        <v>50</v>
       </c>
       <c r="B91" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C91" t="str">
         <f t="shared" si="1"/>
-        <v>BHR6942EU</v>
+        <v>BHR8238EU</v>
       </c>
       <c r="D91" s="3">
-        <v>6941812708347</v>
+        <v>6941812773086</v>
       </c>
       <c r="E91">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F91" t="s">
         <v>7</v>
@@ -2749,20 +2742,20 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="B92" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="C92" t="str">
         <f t="shared" si="1"/>
-        <v>BHR8238EU</v>
+        <v>BHR5274GL</v>
       </c>
       <c r="D92" s="3">
-        <v>6941812773086</v>
+        <v>6934177751158</v>
       </c>
       <c r="E92">
-        <v>53</v>
+        <v>92</v>
       </c>
       <c r="F92" t="s">
         <v>7</v>
@@ -2770,20 +2763,20 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93">
-        <v>120</v>
+        <v>400</v>
       </c>
       <c r="B93" t="s">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="C93" t="str">
         <f t="shared" si="1"/>
-        <v>BHR5274GL</v>
+        <v>BHR8629EU</v>
       </c>
       <c r="D93" s="3">
-        <v>6934177751158</v>
+        <v>6941812786604</v>
       </c>
       <c r="E93">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F93" t="s">
         <v>7</v>
@@ -2791,20 +2784,20 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="B94" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="C94" t="str">
         <f t="shared" si="1"/>
-        <v>BHR5056EU</v>
+        <v>BHR084AEU</v>
       </c>
       <c r="D94" s="3">
-        <v>6934177743665</v>
+        <v>6932554440893</v>
       </c>
       <c r="E94">
-        <v>155</v>
+        <v>99</v>
       </c>
       <c r="F94" t="s">
         <v>7</v>
@@ -2812,20 +2805,20 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="B95" t="s">
-        <v>21</v>
+        <v>92</v>
       </c>
       <c r="C95" t="str">
         <f t="shared" si="1"/>
-        <v>BHR8629EU</v>
+        <v>BHR08GYEU</v>
       </c>
       <c r="D95" s="3">
-        <v>6941812786604</v>
+        <v>6932554458379</v>
       </c>
       <c r="E95">
-        <v>90</v>
+        <v>179</v>
       </c>
       <c r="F95" t="s">
         <v>7</v>
@@ -2833,20 +2826,20 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96">
-        <v>200</v>
+        <v>45</v>
       </c>
       <c r="B96" t="s">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="C96" t="str">
         <f t="shared" si="1"/>
-        <v>BHR084AEU</v>
+        <v>BHR9798EU</v>
       </c>
       <c r="D96" s="3">
-        <v>6932554440893</v>
+        <v>6932554403850</v>
       </c>
       <c r="E96">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="F96" t="s">
         <v>7</v>
@@ -2854,20 +2847,20 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="B97" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C97" t="str">
         <f t="shared" si="1"/>
-        <v>BHR08GYEU</v>
+        <v>BHR5856EU</v>
       </c>
       <c r="D97" s="3">
-        <v>6932554458379</v>
+        <v>6934177775376</v>
       </c>
       <c r="E97">
-        <v>179</v>
+        <v>69</v>
       </c>
       <c r="F97" t="s">
         <v>7</v>
@@ -2875,20 +2868,20 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="B98" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C98" t="str">
         <f t="shared" si="1"/>
-        <v>BHR9798EU</v>
+        <v>ELA6221EU</v>
       </c>
       <c r="D98" s="3">
-        <v>6932554403850</v>
+        <v>6941948706989</v>
       </c>
       <c r="E98">
-        <v>59</v>
+        <v>179</v>
       </c>
       <c r="F98" t="s">
         <v>7</v>
@@ -2896,62 +2889,62 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="B99" t="s">
         <v>94</v>
       </c>
       <c r="C99" t="str">
         <f t="shared" si="1"/>
-        <v>BHR5856EU</v>
+        <v>BHR08OMGL</v>
       </c>
       <c r="D99" s="3">
-        <v>6934177775376</v>
+        <v>6932554471897</v>
       </c>
       <c r="E99">
-        <v>69</v>
+        <v>16</v>
       </c>
       <c r="F99" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="B100" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C100" t="str">
         <f t="shared" si="1"/>
-        <v>ELA6221EU</v>
+        <v>BHR08OLGL</v>
       </c>
       <c r="D100" s="3">
-        <v>6941948706989</v>
+        <v>6932554471880</v>
       </c>
       <c r="E100">
-        <v>179</v>
+        <v>16</v>
       </c>
       <c r="F100" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B101" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C101" t="str">
         <f t="shared" si="1"/>
-        <v>BHR08OMGL</v>
+        <v>BHR07PSGL</v>
       </c>
       <c r="D101" s="3">
-        <v>6932554471897</v>
+        <v>6932554419813</v>
       </c>
       <c r="E101">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F101" t="s">
         <v>6</v>
@@ -2959,20 +2952,20 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B102" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C102" t="str">
         <f t="shared" si="1"/>
-        <v>BHR08OLGL</v>
+        <v>BHR9999GL</v>
       </c>
       <c r="D102" s="3">
-        <v>6932554471880</v>
+        <v>6932554419844</v>
       </c>
       <c r="E102">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F102" t="s">
         <v>6</v>
@@ -2983,17 +2976,17 @@
         <v>90</v>
       </c>
       <c r="B103" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C103" t="str">
         <f t="shared" si="1"/>
-        <v>BHR07PSGL</v>
+        <v>BHR9444GL</v>
       </c>
       <c r="D103" s="3">
-        <v>6932554419813</v>
+        <v>6941812706251</v>
       </c>
       <c r="E103">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F103" t="s">
         <v>6</v>
@@ -3001,20 +2994,20 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="B104" t="s">
-        <v>106</v>
+        <v>11</v>
       </c>
       <c r="C104" t="str">
         <f t="shared" si="1"/>
-        <v>BHR9999GL</v>
+        <v>QBH4380GL</v>
       </c>
       <c r="D104" s="3">
-        <v>6932554419844</v>
+        <v>6941948709218</v>
       </c>
       <c r="E104">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F104" t="s">
         <v>6</v>
@@ -3025,17 +3018,17 @@
         <v>100</v>
       </c>
       <c r="B105" t="s">
-        <v>107</v>
+        <v>12</v>
       </c>
       <c r="C105" t="str">
         <f t="shared" si="1"/>
-        <v>BHR9444GL</v>
+        <v>QBH4378GL</v>
       </c>
       <c r="D105" s="3">
-        <v>6941812706251</v>
+        <v>6941948709201</v>
       </c>
       <c r="E105">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F105" t="s">
         <v>6</v>
@@ -3046,17 +3039,17 @@
         <v>90</v>
       </c>
       <c r="B106" t="s">
-        <v>12</v>
+        <v>115</v>
       </c>
       <c r="C106" t="str">
         <f t="shared" si="1"/>
-        <v>QBH4380GL</v>
+        <v>QBH4265GL</v>
       </c>
       <c r="D106" s="3">
-        <v>6941948709218</v>
+        <v>6941948702042</v>
       </c>
       <c r="E106">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F106" t="s">
         <v>6</v>
@@ -3064,20 +3057,20 @@
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="B107" t="s">
-        <v>13</v>
+        <v>116</v>
       </c>
       <c r="C107" t="str">
         <f t="shared" si="1"/>
-        <v>QBH4378GL</v>
+        <v>QBH4370GL</v>
       </c>
       <c r="D107" s="3">
-        <v>6941948709201</v>
+        <v>6941948709164</v>
       </c>
       <c r="E107">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F107" t="s">
         <v>6</v>
@@ -3085,17 +3078,17 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="B108" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C108" t="str">
         <f t="shared" si="1"/>
-        <v>QBH4265GL</v>
+        <v>QBH4372GL</v>
       </c>
       <c r="D108" s="3">
-        <v>6941948702042</v>
+        <v>6941948709171</v>
       </c>
       <c r="E108">
         <v>28</v>
@@ -3106,17 +3099,17 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="B109" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C109" t="str">
         <f t="shared" si="1"/>
-        <v>QBH4370GL</v>
+        <v>QBH4263GL</v>
       </c>
       <c r="D109" s="3">
-        <v>6941948709164</v>
+        <v>6941948702035</v>
       </c>
       <c r="E109">
         <v>28</v>
@@ -3127,20 +3120,20 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="B110" t="s">
-        <v>121</v>
+        <v>16</v>
       </c>
       <c r="C110" t="str">
         <f t="shared" si="1"/>
-        <v>QBH4372GL</v>
+        <v>QBH2475GL</v>
       </c>
       <c r="D110" s="3">
-        <v>6941948709171</v>
+        <v>6941948703391</v>
       </c>
       <c r="E110">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="F110" t="s">
         <v>6</v>
@@ -3148,20 +3141,20 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="B111" t="s">
-        <v>122</v>
+        <v>13</v>
       </c>
       <c r="C111" t="str">
         <f t="shared" si="1"/>
-        <v>QBH4263GL</v>
+        <v>BHR9073GL</v>
       </c>
       <c r="D111" s="3">
-        <v>6941948702035</v>
+        <v>6941812797501</v>
       </c>
       <c r="E111">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F111" t="s">
         <v>6</v>
@@ -3172,17 +3165,17 @@
         <v>80</v>
       </c>
       <c r="B112" t="s">
+        <v>9</v>
+      </c>
+      <c r="C112" t="str">
+        <f t="shared" si="1"/>
+        <v>BHR9341GL</v>
+      </c>
+      <c r="D112" s="3">
+        <v>6941812774717</v>
+      </c>
+      <c r="E112">
         <v>17</v>
-      </c>
-      <c r="C112" t="str">
-        <f t="shared" si="1"/>
-        <v>QBH2475GL</v>
-      </c>
-      <c r="D112" s="3">
-        <v>6941948703391</v>
-      </c>
-      <c r="E112">
-        <v>38</v>
       </c>
       <c r="F112" t="s">
         <v>6</v>
@@ -3190,20 +3183,20 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="B113" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C113" t="str">
         <f t="shared" si="1"/>
-        <v>BHR9073GL</v>
+        <v>BHR9333GL</v>
       </c>
       <c r="D113" s="3">
-        <v>6941812797501</v>
+        <v>6941812743669</v>
       </c>
       <c r="E113">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F113" t="s">
         <v>6</v>
@@ -3211,20 +3204,20 @@
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B114" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C114" t="str">
         <f t="shared" si="1"/>
-        <v>BHR9341GL</v>
+        <v>BHR8851GL</v>
       </c>
       <c r="D114" s="3">
-        <v>6941812774717</v>
+        <v>6941812792155</v>
       </c>
       <c r="E114">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F114" t="s">
         <v>6</v>
@@ -3232,20 +3225,20 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="B115" t="s">
-        <v>8</v>
+        <v>98</v>
       </c>
       <c r="C115" t="str">
         <f t="shared" si="1"/>
-        <v>BHR9333GL</v>
+        <v>BHR08O8GL</v>
       </c>
       <c r="D115" s="3">
-        <v>6941812743669</v>
+        <v>6932554471194</v>
       </c>
       <c r="E115">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F115" t="s">
         <v>6</v>
@@ -3253,20 +3246,20 @@
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="B116" t="s">
-        <v>28</v>
+        <v>99</v>
       </c>
       <c r="C116" t="str">
         <f t="shared" si="1"/>
-        <v>BHR8851GL</v>
+        <v>BHR08O7GL</v>
       </c>
       <c r="D116" s="3">
-        <v>6941812792155</v>
+        <v>6932554471200</v>
       </c>
       <c r="E116">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F116" t="s">
         <v>6</v>
@@ -3274,20 +3267,20 @@
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="B117" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C117" t="str">
         <f t="shared" si="1"/>
-        <v>BHR08O8GL</v>
+        <v>BHR9970GL</v>
       </c>
       <c r="D117" s="3">
-        <v>6932554471194</v>
+        <v>6932554418410</v>
       </c>
       <c r="E117">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="F117" t="s">
         <v>6</v>
@@ -3295,20 +3288,20 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B118" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C118" t="str">
         <f t="shared" si="1"/>
-        <v>BHR08O7GL</v>
+        <v>BHR08PLGL</v>
       </c>
       <c r="D118" s="3">
-        <v>6932554471200</v>
+        <v>6932554473877</v>
       </c>
       <c r="E118">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F118" t="s">
         <v>6</v>
@@ -3319,17 +3312,17 @@
         <v>10</v>
       </c>
       <c r="B119" t="s">
-        <v>99</v>
+        <v>17</v>
       </c>
       <c r="C119" t="str">
         <f t="shared" si="1"/>
-        <v>BHR9970GL</v>
+        <v>BHR9956EU</v>
       </c>
       <c r="D119" s="3">
-        <v>6932554418410</v>
+        <v>6932554418366</v>
       </c>
       <c r="E119">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="F119" t="s">
         <v>6</v>
@@ -3337,20 +3330,20 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="B120" t="s">
-        <v>108</v>
+        <v>26</v>
       </c>
       <c r="C120" t="str">
         <f t="shared" si="1"/>
-        <v>BHR08PLGL</v>
+        <v>BHR8811EU</v>
       </c>
       <c r="D120" s="3">
-        <v>6932554473877</v>
+        <v>6941812791868</v>
       </c>
       <c r="E120">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F120" t="s">
         <v>6</v>
@@ -3358,20 +3351,20 @@
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B121" t="s">
-        <v>109</v>
+        <v>32</v>
       </c>
       <c r="C121" t="str">
-        <f t="shared" ref="C121:C130" si="2">MID(B121,FIND("@",SUBSTITUTE(B121," ","@",LEN(B121)-LEN(SUBSTITUTE(B121," ",""))))+1,LEN(B121))</f>
-        <v>BHR08Z2GL</v>
+        <f t="shared" si="1"/>
+        <v>BHR9034EU</v>
       </c>
       <c r="D121" s="3">
-        <v>6932554494001</v>
+        <v>6941812796726</v>
       </c>
       <c r="E121">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="F121" t="s">
         <v>6</v>
@@ -3379,20 +3372,20 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B122" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C122" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR9956EU</v>
+        <f t="shared" si="1"/>
+        <v>DVB4514GL</v>
       </c>
       <c r="D122" s="3">
-        <v>6932554418366</v>
+        <v>6941948706736</v>
       </c>
       <c r="E122">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F122" t="s">
         <v>6</v>
@@ -3400,20 +3393,20 @@
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="B123" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="C123" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR8811EU</v>
+        <f t="shared" si="1"/>
+        <v>BHR7456EU</v>
       </c>
       <c r="D123" s="3">
-        <v>6941812791868</v>
+        <v>6941812736579</v>
       </c>
       <c r="E123">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F123" t="s">
         <v>6</v>
@@ -3421,20 +3414,20 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B124" t="s">
-        <v>33</v>
+        <v>93</v>
       </c>
       <c r="C124" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR9034EU</v>
+        <f t="shared" si="1"/>
+        <v>BHR5967EU</v>
       </c>
       <c r="D124" s="3">
-        <v>6941812796726</v>
+        <v>6934177763113</v>
       </c>
       <c r="E124">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F124" t="s">
         <v>6</v>
@@ -3442,20 +3435,20 @@
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B125" t="s">
+        <v>100</v>
+      </c>
+      <c r="C125" t="str">
+        <f t="shared" si="1"/>
+        <v>BHR8955EU</v>
+      </c>
+      <c r="D125" s="3">
+        <v>6941812795941</v>
+      </c>
+      <c r="E125">
         <v>15</v>
-      </c>
-      <c r="C125" t="str">
-        <f t="shared" si="2"/>
-        <v>DVB4514GL</v>
-      </c>
-      <c r="D125" s="3">
-        <v>6941948706736</v>
-      </c>
-      <c r="E125">
-        <v>21</v>
       </c>
       <c r="F125" t="s">
         <v>6</v>
@@ -3463,106 +3456,22 @@
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B126" t="s">
-        <v>11</v>
+        <v>101</v>
       </c>
       <c r="C126" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR7456EU</v>
+        <f t="shared" si="1"/>
+        <v>BHR083KGL</v>
       </c>
       <c r="D126" s="3">
-        <v>6941812736579</v>
+        <v>6932554440435</v>
       </c>
       <c r="E126">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F126" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A127">
-        <v>5</v>
-      </c>
-      <c r="B127" t="s">
-        <v>10</v>
-      </c>
-      <c r="C127" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR7475EU</v>
-      </c>
-      <c r="D127" s="3">
-        <v>6941812736722</v>
-      </c>
-      <c r="E127">
-        <v>15</v>
-      </c>
-      <c r="F127" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A128">
-        <v>50</v>
-      </c>
-      <c r="B128" t="s">
-        <v>96</v>
-      </c>
-      <c r="C128" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR5967EU</v>
-      </c>
-      <c r="D128" s="3">
-        <v>6934177763113</v>
-      </c>
-      <c r="E128">
-        <v>28</v>
-      </c>
-      <c r="F128" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A129">
-        <v>15</v>
-      </c>
-      <c r="B129" t="s">
-        <v>103</v>
-      </c>
-      <c r="C129" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR8955EU</v>
-      </c>
-      <c r="D129" s="3">
-        <v>6941812795941</v>
-      </c>
-      <c r="E129">
-        <v>15</v>
-      </c>
-      <c r="F129" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A130">
-        <v>5</v>
-      </c>
-      <c r="B130" t="s">
-        <v>104</v>
-      </c>
-      <c r="C130" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR083KGL</v>
-      </c>
-      <c r="D130" s="3">
-        <v>6932554440435</v>
-      </c>
-      <c r="E130">
-        <v>12</v>
-      </c>
-      <c r="F130" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>